<commit_message>
Tests with lower bound
</commit_message>
<xml_diff>
--- a/NWJSSP_JuanLlorente_constructivo.xlsx
+++ b/NWJSSP_JuanLlorente_constructivo.xlsx
@@ -20,7 +20,6 @@
     <sheet name="tai_j100_m100_1.txt" sheetId="11" r:id="rId11"/>
     <sheet name="tai_j100_m100_1r.txt" sheetId="12" r:id="rId12"/>
     <sheet name="tai_j1000_m10_1.txt" sheetId="13" r:id="rId13"/>
-    <sheet name="tai_j1000_m10_1r.txt" sheetId="14" r:id="rId14"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1359,7 +1358,7 @@
         <v>573231708</v>
       </c>
       <c r="B1">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:1000">
@@ -4362,3026 +4361,6 @@
       </c>
       <c r="ALL2">
         <v>354469</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:ALL2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:1000">
-      <c r="A1">
-        <v>578273745</v>
-      </c>
-      <c r="B1">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1000">
-      <c r="A2">
-        <v>902757</v>
-      </c>
-      <c r="B2">
-        <v>375279</v>
-      </c>
-      <c r="C2">
-        <v>1191315</v>
-      </c>
-      <c r="D2">
-        <v>271458</v>
-      </c>
-      <c r="E2">
-        <v>579161</v>
-      </c>
-      <c r="F2">
-        <v>888827</v>
-      </c>
-      <c r="G2">
-        <v>1007470</v>
-      </c>
-      <c r="H2">
-        <v>15297</v>
-      </c>
-      <c r="I2">
-        <v>1053319</v>
-      </c>
-      <c r="J2">
-        <v>811743</v>
-      </c>
-      <c r="K2">
-        <v>526521</v>
-      </c>
-      <c r="L2">
-        <v>503617</v>
-      </c>
-      <c r="M2">
-        <v>134927</v>
-      </c>
-      <c r="N2">
-        <v>238876</v>
-      </c>
-      <c r="O2">
-        <v>879434</v>
-      </c>
-      <c r="P2">
-        <v>164167</v>
-      </c>
-      <c r="Q2">
-        <v>1159180</v>
-      </c>
-      <c r="R2">
-        <v>112537</v>
-      </c>
-      <c r="S2">
-        <v>815028</v>
-      </c>
-      <c r="T2">
-        <v>728365</v>
-      </c>
-      <c r="U2">
-        <v>263317</v>
-      </c>
-      <c r="V2">
-        <v>926837</v>
-      </c>
-      <c r="W2">
-        <v>1030631</v>
-      </c>
-      <c r="X2">
-        <v>1194578</v>
-      </c>
-      <c r="Y2">
-        <v>988402</v>
-      </c>
-      <c r="Z2">
-        <v>1309671</v>
-      </c>
-      <c r="AA2">
-        <v>998367</v>
-      </c>
-      <c r="AB2">
-        <v>229334</v>
-      </c>
-      <c r="AC2">
-        <v>196386</v>
-      </c>
-      <c r="AD2">
-        <v>3035</v>
-      </c>
-      <c r="AE2">
-        <v>176230</v>
-      </c>
-      <c r="AF2">
-        <v>600594</v>
-      </c>
-      <c r="AG2">
-        <v>978237</v>
-      </c>
-      <c r="AH2">
-        <v>720616</v>
-      </c>
-      <c r="AI2">
-        <v>1102160</v>
-      </c>
-      <c r="AJ2">
-        <v>748906</v>
-      </c>
-      <c r="AK2">
-        <v>397607</v>
-      </c>
-      <c r="AL2">
-        <v>285213</v>
-      </c>
-      <c r="AM2">
-        <v>630374</v>
-      </c>
-      <c r="AN2">
-        <v>116752</v>
-      </c>
-      <c r="AO2">
-        <v>1285329</v>
-      </c>
-      <c r="AP2">
-        <v>169048</v>
-      </c>
-      <c r="AQ2">
-        <v>138680</v>
-      </c>
-      <c r="AR2">
-        <v>8242</v>
-      </c>
-      <c r="AS2">
-        <v>433312</v>
-      </c>
-      <c r="AT2">
-        <v>343991</v>
-      </c>
-      <c r="AU2">
-        <v>938499</v>
-      </c>
-      <c r="AV2">
-        <v>86209</v>
-      </c>
-      <c r="AW2">
-        <v>294982</v>
-      </c>
-      <c r="AX2">
-        <v>532024</v>
-      </c>
-      <c r="AY2">
-        <v>699253</v>
-      </c>
-      <c r="AZ2">
-        <v>148027</v>
-      </c>
-      <c r="BA2">
-        <v>474648</v>
-      </c>
-      <c r="BB2">
-        <v>98365</v>
-      </c>
-      <c r="BC2">
-        <v>694866</v>
-      </c>
-      <c r="BD2">
-        <v>274259</v>
-      </c>
-      <c r="BE2">
-        <v>314749</v>
-      </c>
-      <c r="BF2">
-        <v>579837</v>
-      </c>
-      <c r="BG2">
-        <v>103144</v>
-      </c>
-      <c r="BH2">
-        <v>131846</v>
-      </c>
-      <c r="BI2">
-        <v>235549</v>
-      </c>
-      <c r="BJ2">
-        <v>300864</v>
-      </c>
-      <c r="BK2">
-        <v>997038</v>
-      </c>
-      <c r="BL2">
-        <v>436827</v>
-      </c>
-      <c r="BM2">
-        <v>542357</v>
-      </c>
-      <c r="BN2">
-        <v>25701</v>
-      </c>
-      <c r="BO2">
-        <v>327419</v>
-      </c>
-      <c r="BP2">
-        <v>77480</v>
-      </c>
-      <c r="BQ2">
-        <v>782363</v>
-      </c>
-      <c r="BR2">
-        <v>948568</v>
-      </c>
-      <c r="BS2">
-        <v>30878</v>
-      </c>
-      <c r="BT2">
-        <v>1061781</v>
-      </c>
-      <c r="BU2">
-        <v>245924</v>
-      </c>
-      <c r="BV2">
-        <v>118821</v>
-      </c>
-      <c r="BW2">
-        <v>55357</v>
-      </c>
-      <c r="BX2">
-        <v>1168619</v>
-      </c>
-      <c r="BY2">
-        <v>133221</v>
-      </c>
-      <c r="BZ2">
-        <v>710609</v>
-      </c>
-      <c r="CA2">
-        <v>953339</v>
-      </c>
-      <c r="CB2">
-        <v>150375</v>
-      </c>
-      <c r="CC2">
-        <v>1211824</v>
-      </c>
-      <c r="CD2">
-        <v>324647</v>
-      </c>
-      <c r="CE2">
-        <v>616014</v>
-      </c>
-      <c r="CF2">
-        <v>596289</v>
-      </c>
-      <c r="CG2">
-        <v>671949</v>
-      </c>
-      <c r="CH2">
-        <v>189942</v>
-      </c>
-      <c r="CI2">
-        <v>647714</v>
-      </c>
-      <c r="CJ2">
-        <v>675128</v>
-      </c>
-      <c r="CK2">
-        <v>740003</v>
-      </c>
-      <c r="CL2">
-        <v>1295419</v>
-      </c>
-      <c r="CM2">
-        <v>659324</v>
-      </c>
-      <c r="CN2">
-        <v>1189523</v>
-      </c>
-      <c r="CO2">
-        <v>1024453</v>
-      </c>
-      <c r="CP2">
-        <v>972119</v>
-      </c>
-      <c r="CQ2">
-        <v>871019</v>
-      </c>
-      <c r="CR2">
-        <v>917101</v>
-      </c>
-      <c r="CS2">
-        <v>68728</v>
-      </c>
-      <c r="CT2">
-        <v>698785</v>
-      </c>
-      <c r="CU2">
-        <v>145338</v>
-      </c>
-      <c r="CV2">
-        <v>792009</v>
-      </c>
-      <c r="CW2">
-        <v>1105104</v>
-      </c>
-      <c r="CX2">
-        <v>656548</v>
-      </c>
-      <c r="CY2">
-        <v>1028271</v>
-      </c>
-      <c r="CZ2">
-        <v>604975</v>
-      </c>
-      <c r="DA2">
-        <v>368948</v>
-      </c>
-      <c r="DB2">
-        <v>568080</v>
-      </c>
-      <c r="DC2">
-        <v>714180</v>
-      </c>
-      <c r="DD2">
-        <v>412198</v>
-      </c>
-      <c r="DE2">
-        <v>52206</v>
-      </c>
-      <c r="DF2">
-        <v>984235</v>
-      </c>
-      <c r="DG2">
-        <v>885982</v>
-      </c>
-      <c r="DH2">
-        <v>95454</v>
-      </c>
-      <c r="DI2">
-        <v>740547</v>
-      </c>
-      <c r="DJ2">
-        <v>1114248</v>
-      </c>
-      <c r="DK2">
-        <v>336286</v>
-      </c>
-      <c r="DL2">
-        <v>397292</v>
-      </c>
-      <c r="DM2">
-        <v>1196333</v>
-      </c>
-      <c r="DN2">
-        <v>1008493</v>
-      </c>
-      <c r="DO2">
-        <v>303627</v>
-      </c>
-      <c r="DP2">
-        <v>961733</v>
-      </c>
-      <c r="DQ2">
-        <v>893247</v>
-      </c>
-      <c r="DR2">
-        <v>856325</v>
-      </c>
-      <c r="DS2">
-        <v>639609</v>
-      </c>
-      <c r="DT2">
-        <v>394562</v>
-      </c>
-      <c r="DU2">
-        <v>341815</v>
-      </c>
-      <c r="DV2">
-        <v>1043945</v>
-      </c>
-      <c r="DW2">
-        <v>414930</v>
-      </c>
-      <c r="DX2">
-        <v>371180</v>
-      </c>
-      <c r="DY2">
-        <v>1186364</v>
-      </c>
-      <c r="DZ2">
-        <v>1108012</v>
-      </c>
-      <c r="EA2">
-        <v>762271</v>
-      </c>
-      <c r="EB2">
-        <v>1012714</v>
-      </c>
-      <c r="EC2">
-        <v>50299</v>
-      </c>
-      <c r="ED2">
-        <v>831483</v>
-      </c>
-      <c r="EE2">
-        <v>285362</v>
-      </c>
-      <c r="EF2">
-        <v>282674</v>
-      </c>
-      <c r="EG2">
-        <v>277887</v>
-      </c>
-      <c r="EH2">
-        <v>299655</v>
-      </c>
-      <c r="EI2">
-        <v>1082196</v>
-      </c>
-      <c r="EJ2">
-        <v>305388</v>
-      </c>
-      <c r="EK2">
-        <v>72853</v>
-      </c>
-      <c r="EL2">
-        <v>683764</v>
-      </c>
-      <c r="EM2">
-        <v>178363</v>
-      </c>
-      <c r="EN2">
-        <v>683356</v>
-      </c>
-      <c r="EO2">
-        <v>531272</v>
-      </c>
-      <c r="EP2">
-        <v>160886</v>
-      </c>
-      <c r="EQ2">
-        <v>534951</v>
-      </c>
-      <c r="ER2">
-        <v>311629</v>
-      </c>
-      <c r="ES2">
-        <v>663182</v>
-      </c>
-      <c r="ET2">
-        <v>198776</v>
-      </c>
-      <c r="EU2">
-        <v>896229</v>
-      </c>
-      <c r="EV2">
-        <v>947276</v>
-      </c>
-      <c r="EW2">
-        <v>204690</v>
-      </c>
-      <c r="EX2">
-        <v>827360</v>
-      </c>
-      <c r="EY2">
-        <v>1010962</v>
-      </c>
-      <c r="EZ2">
-        <v>164861</v>
-      </c>
-      <c r="FA2">
-        <v>191426</v>
-      </c>
-      <c r="FB2">
-        <v>826374</v>
-      </c>
-      <c r="FC2">
-        <v>990742</v>
-      </c>
-      <c r="FD2">
-        <v>640569</v>
-      </c>
-      <c r="FE2">
-        <v>976891</v>
-      </c>
-      <c r="FF2">
-        <v>70861</v>
-      </c>
-      <c r="FG2">
-        <v>931063</v>
-      </c>
-      <c r="FH2">
-        <v>725993</v>
-      </c>
-      <c r="FI2">
-        <v>1111656</v>
-      </c>
-      <c r="FJ2">
-        <v>965193</v>
-      </c>
-      <c r="FK2">
-        <v>505435</v>
-      </c>
-      <c r="FL2">
-        <v>817450</v>
-      </c>
-      <c r="FM2">
-        <v>636790</v>
-      </c>
-      <c r="FN2">
-        <v>37299</v>
-      </c>
-      <c r="FO2">
-        <v>685002</v>
-      </c>
-      <c r="FP2">
-        <v>170933</v>
-      </c>
-      <c r="FQ2">
-        <v>45664</v>
-      </c>
-      <c r="FR2">
-        <v>617852</v>
-      </c>
-      <c r="FS2">
-        <v>226813</v>
-      </c>
-      <c r="FT2">
-        <v>497125</v>
-      </c>
-      <c r="FU2">
-        <v>352915</v>
-      </c>
-      <c r="FV2">
-        <v>358905</v>
-      </c>
-      <c r="FW2">
-        <v>456551</v>
-      </c>
-      <c r="FX2">
-        <v>429600</v>
-      </c>
-      <c r="FY2">
-        <v>942068</v>
-      </c>
-      <c r="FZ2">
-        <v>335945</v>
-      </c>
-      <c r="GA2">
-        <v>491048</v>
-      </c>
-      <c r="GB2">
-        <v>795458</v>
-      </c>
-      <c r="GC2">
-        <v>1015863</v>
-      </c>
-      <c r="GD2">
-        <v>494455</v>
-      </c>
-      <c r="GE2">
-        <v>612816</v>
-      </c>
-      <c r="GF2">
-        <v>99140</v>
-      </c>
-      <c r="GG2">
-        <v>935523</v>
-      </c>
-      <c r="GH2">
-        <v>692066</v>
-      </c>
-      <c r="GI2">
-        <v>594131</v>
-      </c>
-      <c r="GJ2">
-        <v>699391</v>
-      </c>
-      <c r="GK2">
-        <v>23350</v>
-      </c>
-      <c r="GL2">
-        <v>861031</v>
-      </c>
-      <c r="GM2">
-        <v>797733</v>
-      </c>
-      <c r="GN2">
-        <v>521930</v>
-      </c>
-      <c r="GO2">
-        <v>109244</v>
-      </c>
-      <c r="GP2">
-        <v>363862</v>
-      </c>
-      <c r="GQ2">
-        <v>23588</v>
-      </c>
-      <c r="GR2">
-        <v>23157</v>
-      </c>
-      <c r="GS2">
-        <v>969988</v>
-      </c>
-      <c r="GT2">
-        <v>851239</v>
-      </c>
-      <c r="GU2">
-        <v>1038676</v>
-      </c>
-      <c r="GV2">
-        <v>252915</v>
-      </c>
-      <c r="GW2">
-        <v>348274</v>
-      </c>
-      <c r="GX2">
-        <v>673089</v>
-      </c>
-      <c r="GY2">
-        <v>407780</v>
-      </c>
-      <c r="GZ2">
-        <v>47817</v>
-      </c>
-      <c r="HA2">
-        <v>765730</v>
-      </c>
-      <c r="HB2">
-        <v>280970</v>
-      </c>
-      <c r="HC2">
-        <v>437078</v>
-      </c>
-      <c r="HD2">
-        <v>918570</v>
-      </c>
-      <c r="HE2">
-        <v>1045568</v>
-      </c>
-      <c r="HF2">
-        <v>645573</v>
-      </c>
-      <c r="HG2">
-        <v>235114</v>
-      </c>
-      <c r="HH2">
-        <v>128877</v>
-      </c>
-      <c r="HI2">
-        <v>1071703</v>
-      </c>
-      <c r="HJ2">
-        <v>626297</v>
-      </c>
-      <c r="HK2">
-        <v>805360</v>
-      </c>
-      <c r="HL2">
-        <v>888650</v>
-      </c>
-      <c r="HM2">
-        <v>770257</v>
-      </c>
-      <c r="HN2">
-        <v>1068949</v>
-      </c>
-      <c r="HO2">
-        <v>1280864</v>
-      </c>
-      <c r="HP2">
-        <v>871531</v>
-      </c>
-      <c r="HQ2">
-        <v>1092150</v>
-      </c>
-      <c r="HR2">
-        <v>560594</v>
-      </c>
-      <c r="HS2">
-        <v>1005721</v>
-      </c>
-      <c r="HT2">
-        <v>838378</v>
-      </c>
-      <c r="HU2">
-        <v>305381</v>
-      </c>
-      <c r="HV2">
-        <v>805100</v>
-      </c>
-      <c r="HW2">
-        <v>55973</v>
-      </c>
-      <c r="HX2">
-        <v>400595</v>
-      </c>
-      <c r="HY2">
-        <v>876285</v>
-      </c>
-      <c r="HZ2">
-        <v>110769</v>
-      </c>
-      <c r="IA2">
-        <v>1217022</v>
-      </c>
-      <c r="IB2">
-        <v>1078336</v>
-      </c>
-      <c r="IC2">
-        <v>754192</v>
-      </c>
-      <c r="ID2">
-        <v>1094747</v>
-      </c>
-      <c r="IE2">
-        <v>515009</v>
-      </c>
-      <c r="IF2">
-        <v>70008</v>
-      </c>
-      <c r="IG2">
-        <v>364</v>
-      </c>
-      <c r="IH2">
-        <v>761286</v>
-      </c>
-      <c r="II2">
-        <v>79881</v>
-      </c>
-      <c r="IJ2">
-        <v>193731</v>
-      </c>
-      <c r="IK2">
-        <v>910049</v>
-      </c>
-      <c r="IL2">
-        <v>540905</v>
-      </c>
-      <c r="IM2">
-        <v>993306</v>
-      </c>
-      <c r="IN2">
-        <v>645091</v>
-      </c>
-      <c r="IO2">
-        <v>145038</v>
-      </c>
-      <c r="IP2">
-        <v>180777</v>
-      </c>
-      <c r="IQ2">
-        <v>1022664</v>
-      </c>
-      <c r="IR2">
-        <v>1224254</v>
-      </c>
-      <c r="IS2">
-        <v>881924</v>
-      </c>
-      <c r="IT2">
-        <v>1290667</v>
-      </c>
-      <c r="IU2">
-        <v>1207551</v>
-      </c>
-      <c r="IV2">
-        <v>831155</v>
-      </c>
-      <c r="IW2">
-        <v>273812</v>
-      </c>
-      <c r="IX2">
-        <v>202205</v>
-      </c>
-      <c r="IY2">
-        <v>834623</v>
-      </c>
-      <c r="IZ2">
-        <v>40087</v>
-      </c>
-      <c r="JA2">
-        <v>566644</v>
-      </c>
-      <c r="JB2">
-        <v>292654</v>
-      </c>
-      <c r="JC2">
-        <v>1086277</v>
-      </c>
-      <c r="JD2">
-        <v>1130238</v>
-      </c>
-      <c r="JE2">
-        <v>732467</v>
-      </c>
-      <c r="JF2">
-        <v>261622</v>
-      </c>
-      <c r="JG2">
-        <v>134317</v>
-      </c>
-      <c r="JH2">
-        <v>288222</v>
-      </c>
-      <c r="JI2">
-        <v>85435</v>
-      </c>
-      <c r="JJ2">
-        <v>776535</v>
-      </c>
-      <c r="JK2">
-        <v>768041</v>
-      </c>
-      <c r="JL2">
-        <v>1280935</v>
-      </c>
-      <c r="JM2">
-        <v>44174</v>
-      </c>
-      <c r="JN2">
-        <v>351236</v>
-      </c>
-      <c r="JO2">
-        <v>1054640</v>
-      </c>
-      <c r="JP2">
-        <v>659308</v>
-      </c>
-      <c r="JQ2">
-        <v>814649</v>
-      </c>
-      <c r="JR2">
-        <v>649825</v>
-      </c>
-      <c r="JS2">
-        <v>970976</v>
-      </c>
-      <c r="JT2">
-        <v>1200301</v>
-      </c>
-      <c r="JU2">
-        <v>391085</v>
-      </c>
-      <c r="JV2">
-        <v>312760</v>
-      </c>
-      <c r="JW2">
-        <v>415164</v>
-      </c>
-      <c r="JX2">
-        <v>851396</v>
-      </c>
-      <c r="JY2">
-        <v>422263</v>
-      </c>
-      <c r="JZ2">
-        <v>394344</v>
-      </c>
-      <c r="KA2">
-        <v>960503</v>
-      </c>
-      <c r="KB2">
-        <v>86620</v>
-      </c>
-      <c r="KC2">
-        <v>177605</v>
-      </c>
-      <c r="KD2">
-        <v>88989</v>
-      </c>
-      <c r="KE2">
-        <v>745059</v>
-      </c>
-      <c r="KF2">
-        <v>440755</v>
-      </c>
-      <c r="KG2">
-        <v>214163</v>
-      </c>
-      <c r="KH2">
-        <v>210580</v>
-      </c>
-      <c r="KI2">
-        <v>163307</v>
-      </c>
-      <c r="KJ2">
-        <v>923281</v>
-      </c>
-      <c r="KK2">
-        <v>1297213</v>
-      </c>
-      <c r="KL2">
-        <v>318928</v>
-      </c>
-      <c r="KM2">
-        <v>452160</v>
-      </c>
-      <c r="KN2">
-        <v>239382</v>
-      </c>
-      <c r="KO2">
-        <v>1137465</v>
-      </c>
-      <c r="KP2">
-        <v>341282</v>
-      </c>
-      <c r="KQ2">
-        <v>187367</v>
-      </c>
-      <c r="KR2">
-        <v>862525</v>
-      </c>
-      <c r="KS2">
-        <v>931799</v>
-      </c>
-      <c r="KT2">
-        <v>210117</v>
-      </c>
-      <c r="KU2">
-        <v>723212</v>
-      </c>
-      <c r="KV2">
-        <v>803153</v>
-      </c>
-      <c r="KW2">
-        <v>314458</v>
-      </c>
-      <c r="KX2">
-        <v>1035620</v>
-      </c>
-      <c r="KY2">
-        <v>1131117</v>
-      </c>
-      <c r="KZ2">
-        <v>610905</v>
-      </c>
-      <c r="LA2">
-        <v>79566</v>
-      </c>
-      <c r="LB2">
-        <v>547213</v>
-      </c>
-      <c r="LC2">
-        <v>491945</v>
-      </c>
-      <c r="LD2">
-        <v>755231</v>
-      </c>
-      <c r="LE2">
-        <v>1247292</v>
-      </c>
-      <c r="LF2">
-        <v>355656</v>
-      </c>
-      <c r="LG2">
-        <v>804868</v>
-      </c>
-      <c r="LH2">
-        <v>352665</v>
-      </c>
-      <c r="LI2">
-        <v>224375</v>
-      </c>
-      <c r="LJ2">
-        <v>1143848</v>
-      </c>
-      <c r="LK2">
-        <v>1205021</v>
-      </c>
-      <c r="LL2">
-        <v>612424</v>
-      </c>
-      <c r="LM2">
-        <v>753234</v>
-      </c>
-      <c r="LN2">
-        <v>392657</v>
-      </c>
-      <c r="LO2">
-        <v>124840</v>
-      </c>
-      <c r="LP2">
-        <v>612160</v>
-      </c>
-      <c r="LQ2">
-        <v>590322</v>
-      </c>
-      <c r="LR2">
-        <v>636065</v>
-      </c>
-      <c r="LS2">
-        <v>169712</v>
-      </c>
-      <c r="LT2">
-        <v>239994</v>
-      </c>
-      <c r="LU2">
-        <v>923718</v>
-      </c>
-      <c r="LV2">
-        <v>1077830</v>
-      </c>
-      <c r="LW2">
-        <v>1253536</v>
-      </c>
-      <c r="LX2">
-        <v>421011</v>
-      </c>
-      <c r="LY2">
-        <v>528377</v>
-      </c>
-      <c r="LZ2">
-        <v>1002591</v>
-      </c>
-      <c r="MA2">
-        <v>786395</v>
-      </c>
-      <c r="MB2">
-        <v>897729</v>
-      </c>
-      <c r="MC2">
-        <v>678122</v>
-      </c>
-      <c r="MD2">
-        <v>58688</v>
-      </c>
-      <c r="ME2">
-        <v>825386</v>
-      </c>
-      <c r="MF2">
-        <v>331750</v>
-      </c>
-      <c r="MG2">
-        <v>1059474</v>
-      </c>
-      <c r="MH2">
-        <v>467074</v>
-      </c>
-      <c r="MI2">
-        <v>965414</v>
-      </c>
-      <c r="MJ2">
-        <v>413848</v>
-      </c>
-      <c r="MK2">
-        <v>410423</v>
-      </c>
-      <c r="ML2">
-        <v>290855</v>
-      </c>
-      <c r="MM2">
-        <v>116926</v>
-      </c>
-      <c r="MN2">
-        <v>562609</v>
-      </c>
-      <c r="MO2">
-        <v>222008</v>
-      </c>
-      <c r="MP2">
-        <v>560262</v>
-      </c>
-      <c r="MQ2">
-        <v>808611</v>
-      </c>
-      <c r="MR2">
-        <v>143155</v>
-      </c>
-      <c r="MS2">
-        <v>902658</v>
-      </c>
-      <c r="MT2">
-        <v>663746</v>
-      </c>
-      <c r="MU2">
-        <v>166181</v>
-      </c>
-      <c r="MV2">
-        <v>921517</v>
-      </c>
-      <c r="MW2">
-        <v>617932</v>
-      </c>
-      <c r="MX2">
-        <v>891665</v>
-      </c>
-      <c r="MY2">
-        <v>8827</v>
-      </c>
-      <c r="MZ2">
-        <v>1161965</v>
-      </c>
-      <c r="NA2">
-        <v>1017324</v>
-      </c>
-      <c r="NB2">
-        <v>1234161</v>
-      </c>
-      <c r="NC2">
-        <v>550349</v>
-      </c>
-      <c r="ND2">
-        <v>1096896</v>
-      </c>
-      <c r="NE2">
-        <v>555658</v>
-      </c>
-      <c r="NF2">
-        <v>318070</v>
-      </c>
-      <c r="NG2">
-        <v>214702</v>
-      </c>
-      <c r="NH2">
-        <v>572147</v>
-      </c>
-      <c r="NI2">
-        <v>465447</v>
-      </c>
-      <c r="NJ2">
-        <v>1101178</v>
-      </c>
-      <c r="NK2">
-        <v>244959</v>
-      </c>
-      <c r="NL2">
-        <v>1016537</v>
-      </c>
-      <c r="NM2">
-        <v>256686</v>
-      </c>
-      <c r="NN2">
-        <v>479250</v>
-      </c>
-      <c r="NO2">
-        <v>111865</v>
-      </c>
-      <c r="NP2">
-        <v>224718</v>
-      </c>
-      <c r="NQ2">
-        <v>346133</v>
-      </c>
-      <c r="NR2">
-        <v>444787</v>
-      </c>
-      <c r="NS2">
-        <v>209602</v>
-      </c>
-      <c r="NT2">
-        <v>1058742</v>
-      </c>
-      <c r="NU2">
-        <v>267332</v>
-      </c>
-      <c r="NV2">
-        <v>470715</v>
-      </c>
-      <c r="NW2">
-        <v>10090</v>
-      </c>
-      <c r="NX2">
-        <v>1077</v>
-      </c>
-      <c r="NY2">
-        <v>259912</v>
-      </c>
-      <c r="NZ2">
-        <v>835070</v>
-      </c>
-      <c r="OA2">
-        <v>192239</v>
-      </c>
-      <c r="OB2">
-        <v>190413</v>
-      </c>
-      <c r="OC2">
-        <v>234824</v>
-      </c>
-      <c r="OD2">
-        <v>651317</v>
-      </c>
-      <c r="OE2">
-        <v>359644</v>
-      </c>
-      <c r="OF2">
-        <v>624046</v>
-      </c>
-      <c r="OG2">
-        <v>13168</v>
-      </c>
-      <c r="OH2">
-        <v>942686</v>
-      </c>
-      <c r="OI2">
-        <v>505606</v>
-      </c>
-      <c r="OJ2">
-        <v>687664</v>
-      </c>
-      <c r="OK2">
-        <v>593136</v>
-      </c>
-      <c r="OL2">
-        <v>499268</v>
-      </c>
-      <c r="OM2">
-        <v>666426</v>
-      </c>
-      <c r="ON2">
-        <v>331330</v>
-      </c>
-      <c r="OO2">
-        <v>876993</v>
-      </c>
-      <c r="OP2">
-        <v>518433</v>
-      </c>
-      <c r="OQ2">
-        <v>156795</v>
-      </c>
-      <c r="OR2">
-        <v>1050753</v>
-      </c>
-      <c r="OS2">
-        <v>873779</v>
-      </c>
-      <c r="OT2">
-        <v>118440</v>
-      </c>
-      <c r="OU2">
-        <v>869040</v>
-      </c>
-      <c r="OV2">
-        <v>793329</v>
-      </c>
-      <c r="OW2">
-        <v>778303</v>
-      </c>
-      <c r="OX2">
-        <v>1116308</v>
-      </c>
-      <c r="OY2">
-        <v>200261</v>
-      </c>
-      <c r="OZ2">
-        <v>701596</v>
-      </c>
-      <c r="PA2">
-        <v>1066685</v>
-      </c>
-      <c r="PB2">
-        <v>1081144</v>
-      </c>
-      <c r="PC2">
-        <v>470117</v>
-      </c>
-      <c r="PD2">
-        <v>401252</v>
-      </c>
-      <c r="PE2">
-        <v>1106517</v>
-      </c>
-      <c r="PF2">
-        <v>601127</v>
-      </c>
-      <c r="PG2">
-        <v>443722</v>
-      </c>
-      <c r="PH2">
-        <v>640153</v>
-      </c>
-      <c r="PI2">
-        <v>600907</v>
-      </c>
-      <c r="PJ2">
-        <v>42671</v>
-      </c>
-      <c r="PK2">
-        <v>128197</v>
-      </c>
-      <c r="PL2">
-        <v>454790</v>
-      </c>
-      <c r="PM2">
-        <v>294425</v>
-      </c>
-      <c r="PN2">
-        <v>0</v>
-      </c>
-      <c r="PO2">
-        <v>1177124</v>
-      </c>
-      <c r="PP2">
-        <v>482744</v>
-      </c>
-      <c r="PQ2">
-        <v>722133</v>
-      </c>
-      <c r="PR2">
-        <v>689016</v>
-      </c>
-      <c r="PS2">
-        <v>788008</v>
-      </c>
-      <c r="PT2">
-        <v>327946</v>
-      </c>
-      <c r="PU2">
-        <v>52667</v>
-      </c>
-      <c r="PV2">
-        <v>272331</v>
-      </c>
-      <c r="PW2">
-        <v>275364</v>
-      </c>
-      <c r="PX2">
-        <v>260147</v>
-      </c>
-      <c r="PY2">
-        <v>248691</v>
-      </c>
-      <c r="PZ2">
-        <v>416283</v>
-      </c>
-      <c r="QA2">
-        <v>389678</v>
-      </c>
-      <c r="QB2">
-        <v>374185</v>
-      </c>
-      <c r="QC2">
-        <v>125164</v>
-      </c>
-      <c r="QD2">
-        <v>95401</v>
-      </c>
-      <c r="QE2">
-        <v>568991</v>
-      </c>
-      <c r="QF2">
-        <v>342774</v>
-      </c>
-      <c r="QG2">
-        <v>159570</v>
-      </c>
-      <c r="QH2">
-        <v>1140601</v>
-      </c>
-      <c r="QI2">
-        <v>409139</v>
-      </c>
-      <c r="QJ2">
-        <v>881070</v>
-      </c>
-      <c r="QK2">
-        <v>11589</v>
-      </c>
-      <c r="QL2">
-        <v>854748</v>
-      </c>
-      <c r="QM2">
-        <v>1222541</v>
-      </c>
-      <c r="QN2">
-        <v>368716</v>
-      </c>
-      <c r="QO2">
-        <v>39606</v>
-      </c>
-      <c r="QP2">
-        <v>7752</v>
-      </c>
-      <c r="QQ2">
-        <v>501047</v>
-      </c>
-      <c r="QR2">
-        <v>364521</v>
-      </c>
-      <c r="QS2">
-        <v>1155426</v>
-      </c>
-      <c r="QT2">
-        <v>792813</v>
-      </c>
-      <c r="QU2">
-        <v>575308</v>
-      </c>
-      <c r="QV2">
-        <v>1304323</v>
-      </c>
-      <c r="QW2">
-        <v>61493</v>
-      </c>
-      <c r="QX2">
-        <v>819405</v>
-      </c>
-      <c r="QY2">
-        <v>1143447</v>
-      </c>
-      <c r="QZ2">
-        <v>1167839</v>
-      </c>
-      <c r="RA2">
-        <v>174963</v>
-      </c>
-      <c r="RB2">
-        <v>736548</v>
-      </c>
-      <c r="RC2">
-        <v>67562</v>
-      </c>
-      <c r="RD2">
-        <v>1032543</v>
-      </c>
-      <c r="RE2">
-        <v>58100</v>
-      </c>
-      <c r="RF2">
-        <v>448389</v>
-      </c>
-      <c r="RG2">
-        <v>373888</v>
-      </c>
-      <c r="RH2">
-        <v>507616</v>
-      </c>
-      <c r="RI2">
-        <v>309775</v>
-      </c>
-      <c r="RJ2">
-        <v>733658</v>
-      </c>
-      <c r="RK2">
-        <v>1244085</v>
-      </c>
-      <c r="RL2">
-        <v>1302230</v>
-      </c>
-      <c r="RM2">
-        <v>564847</v>
-      </c>
-      <c r="RN2">
-        <v>263223</v>
-      </c>
-      <c r="RO2">
-        <v>114231</v>
-      </c>
-      <c r="RP2">
-        <v>701171</v>
-      </c>
-      <c r="RQ2">
-        <v>543513</v>
-      </c>
-      <c r="RR2">
-        <v>711557</v>
-      </c>
-      <c r="RS2">
-        <v>1066000</v>
-      </c>
-      <c r="RT2">
-        <v>101705</v>
-      </c>
-      <c r="RU2">
-        <v>49493</v>
-      </c>
-      <c r="RV2">
-        <v>212491</v>
-      </c>
-      <c r="RW2">
-        <v>459186</v>
-      </c>
-      <c r="RX2">
-        <v>241756</v>
-      </c>
-      <c r="RY2">
-        <v>1184604</v>
-      </c>
-      <c r="RZ2">
-        <v>1140565</v>
-      </c>
-      <c r="SA2">
-        <v>257435</v>
-      </c>
-      <c r="SB2">
-        <v>358000</v>
-      </c>
-      <c r="SC2">
-        <v>712043</v>
-      </c>
-      <c r="SD2">
-        <v>75094</v>
-      </c>
-      <c r="SE2">
-        <v>501027</v>
-      </c>
-      <c r="SF2">
-        <v>1152080</v>
-      </c>
-      <c r="SG2">
-        <v>1048494</v>
-      </c>
-      <c r="SH2">
-        <v>394365</v>
-      </c>
-      <c r="SI2">
-        <v>27302</v>
-      </c>
-      <c r="SJ2">
-        <v>709777</v>
-      </c>
-      <c r="SK2">
-        <v>464788</v>
-      </c>
-      <c r="SL2">
-        <v>406689</v>
-      </c>
-      <c r="SM2">
-        <v>319663</v>
-      </c>
-      <c r="SN2">
-        <v>617667</v>
-      </c>
-      <c r="SO2">
-        <v>151951</v>
-      </c>
-      <c r="SP2">
-        <v>933167</v>
-      </c>
-      <c r="SQ2">
-        <v>892194</v>
-      </c>
-      <c r="SR2">
-        <v>13843</v>
-      </c>
-      <c r="SS2">
-        <v>694213</v>
-      </c>
-      <c r="ST2">
-        <v>685302</v>
-      </c>
-      <c r="SU2">
-        <v>254509</v>
-      </c>
-      <c r="SV2">
-        <v>652738</v>
-      </c>
-      <c r="SW2">
-        <v>308966</v>
-      </c>
-      <c r="SX2">
-        <v>911105</v>
-      </c>
-      <c r="SY2">
-        <v>1153580</v>
-      </c>
-      <c r="SZ2">
-        <v>1097806</v>
-      </c>
-      <c r="TA2">
-        <v>780932</v>
-      </c>
-      <c r="TB2">
-        <v>1012347</v>
-      </c>
-      <c r="TC2">
-        <v>12883</v>
-      </c>
-      <c r="TD2">
-        <v>913669</v>
-      </c>
-      <c r="TE2">
-        <v>1072522</v>
-      </c>
-      <c r="TF2">
-        <v>430416</v>
-      </c>
-      <c r="TG2">
-        <v>355664</v>
-      </c>
-      <c r="TH2">
-        <v>217360</v>
-      </c>
-      <c r="TI2">
-        <v>726652</v>
-      </c>
-      <c r="TJ2">
-        <v>148498</v>
-      </c>
-      <c r="TK2">
-        <v>370252</v>
-      </c>
-      <c r="TL2">
-        <v>33515</v>
-      </c>
-      <c r="TM2">
-        <v>268989</v>
-      </c>
-      <c r="TN2">
-        <v>168150</v>
-      </c>
-      <c r="TO2">
-        <v>27152</v>
-      </c>
-      <c r="TP2">
-        <v>418574</v>
-      </c>
-      <c r="TQ2">
-        <v>437900</v>
-      </c>
-      <c r="TR2">
-        <v>21288</v>
-      </c>
-      <c r="TS2">
-        <v>1103495</v>
-      </c>
-      <c r="TT2">
-        <v>218923</v>
-      </c>
-      <c r="TU2">
-        <v>552550</v>
-      </c>
-      <c r="TV2">
-        <v>954107</v>
-      </c>
-      <c r="TW2">
-        <v>293974</v>
-      </c>
-      <c r="TX2">
-        <v>35416</v>
-      </c>
-      <c r="TY2">
-        <v>762307</v>
-      </c>
-      <c r="TZ2">
-        <v>475414</v>
-      </c>
-      <c r="UA2">
-        <v>1301154</v>
-      </c>
-      <c r="UB2">
-        <v>385108</v>
-      </c>
-      <c r="UC2">
-        <v>846596</v>
-      </c>
-      <c r="UD2">
-        <v>448616</v>
-      </c>
-      <c r="UE2">
-        <v>53443</v>
-      </c>
-      <c r="UF2">
-        <v>606875</v>
-      </c>
-      <c r="UG2">
-        <v>83811</v>
-      </c>
-      <c r="UH2">
-        <v>322427</v>
-      </c>
-      <c r="UI2">
-        <v>1175628</v>
-      </c>
-      <c r="UJ2">
-        <v>488773</v>
-      </c>
-      <c r="UK2">
-        <v>855998</v>
-      </c>
-      <c r="UL2">
-        <v>545586</v>
-      </c>
-      <c r="UM2">
-        <v>1230182</v>
-      </c>
-      <c r="UN2">
-        <v>1269402</v>
-      </c>
-      <c r="UO2">
-        <v>799043</v>
-      </c>
-      <c r="UP2">
-        <v>640034</v>
-      </c>
-      <c r="UQ2">
-        <v>1120556</v>
-      </c>
-      <c r="UR2">
-        <v>964253</v>
-      </c>
-      <c r="US2">
-        <v>138806</v>
-      </c>
-      <c r="UT2">
-        <v>623865</v>
-      </c>
-      <c r="UU2">
-        <v>1235773</v>
-      </c>
-      <c r="UV2">
-        <v>841049</v>
-      </c>
-      <c r="UW2">
-        <v>576963</v>
-      </c>
-      <c r="UX2">
-        <v>444786</v>
-      </c>
-      <c r="UY2">
-        <v>172992</v>
-      </c>
-      <c r="UZ2">
-        <v>1031258</v>
-      </c>
-      <c r="VA2">
-        <v>1286471</v>
-      </c>
-      <c r="VB2">
-        <v>900316</v>
-      </c>
-      <c r="VC2">
-        <v>386713</v>
-      </c>
-      <c r="VD2">
-        <v>1174359</v>
-      </c>
-      <c r="VE2">
-        <v>1248235</v>
-      </c>
-      <c r="VF2">
-        <v>473457</v>
-      </c>
-      <c r="VG2">
-        <v>380032</v>
-      </c>
-      <c r="VH2">
-        <v>154469</v>
-      </c>
-      <c r="VI2">
-        <v>1136368</v>
-      </c>
-      <c r="VJ2">
-        <v>1122940</v>
-      </c>
-      <c r="VK2">
-        <v>93664</v>
-      </c>
-      <c r="VL2">
-        <v>675974</v>
-      </c>
-      <c r="VM2">
-        <v>387358</v>
-      </c>
-      <c r="VN2">
-        <v>326945</v>
-      </c>
-      <c r="VO2">
-        <v>603534</v>
-      </c>
-      <c r="VP2">
-        <v>289515</v>
-      </c>
-      <c r="VQ2">
-        <v>140891</v>
-      </c>
-      <c r="VR2">
-        <v>850557</v>
-      </c>
-      <c r="VS2">
-        <v>9622</v>
-      </c>
-      <c r="VT2">
-        <v>381800</v>
-      </c>
-      <c r="VU2">
-        <v>156611</v>
-      </c>
-      <c r="VV2">
-        <v>848256</v>
-      </c>
-      <c r="VW2">
-        <v>560689</v>
-      </c>
-      <c r="VX2">
-        <v>1292865</v>
-      </c>
-      <c r="VY2">
-        <v>496205</v>
-      </c>
-      <c r="VZ2">
-        <v>65902</v>
-      </c>
-      <c r="WA2">
-        <v>1148192</v>
-      </c>
-      <c r="WB2">
-        <v>184202</v>
-      </c>
-      <c r="WC2">
-        <v>1037568</v>
-      </c>
-      <c r="WD2">
-        <v>945488</v>
-      </c>
-      <c r="WE2">
-        <v>695712</v>
-      </c>
-      <c r="WF2">
-        <v>1226533</v>
-      </c>
-      <c r="WG2">
-        <v>668002</v>
-      </c>
-      <c r="WH2">
-        <v>669592</v>
-      </c>
-      <c r="WI2">
-        <v>680526</v>
-      </c>
-      <c r="WJ2">
-        <v>633066</v>
-      </c>
-      <c r="WK2">
-        <v>1195099</v>
-      </c>
-      <c r="WL2">
-        <v>182031</v>
-      </c>
-      <c r="WM2">
-        <v>58968</v>
-      </c>
-      <c r="WN2">
-        <v>140419</v>
-      </c>
-      <c r="WO2">
-        <v>1173133</v>
-      </c>
-      <c r="WP2">
-        <v>2368</v>
-      </c>
-      <c r="WQ2">
-        <v>800278</v>
-      </c>
-      <c r="WR2">
-        <v>525911</v>
-      </c>
-      <c r="WS2">
-        <v>879254</v>
-      </c>
-      <c r="WT2">
-        <v>30217</v>
-      </c>
-      <c r="WU2">
-        <v>1126896</v>
-      </c>
-      <c r="WV2">
-        <v>76797</v>
-      </c>
-      <c r="WW2">
-        <v>250565</v>
-      </c>
-      <c r="WX2">
-        <v>537924</v>
-      </c>
-      <c r="WY2">
-        <v>241661</v>
-      </c>
-      <c r="WZ2">
-        <v>72044</v>
-      </c>
-      <c r="XA2">
-        <v>517448</v>
-      </c>
-      <c r="XB2">
-        <v>135578</v>
-      </c>
-      <c r="XC2">
-        <v>751922</v>
-      </c>
-      <c r="XD2">
-        <v>1092203</v>
-      </c>
-      <c r="XE2">
-        <v>325082</v>
-      </c>
-      <c r="XF2">
-        <v>420225</v>
-      </c>
-      <c r="XG2">
-        <v>1259054</v>
-      </c>
-      <c r="XH2">
-        <v>859839</v>
-      </c>
-      <c r="XI2">
-        <v>224862</v>
-      </c>
-      <c r="XJ2">
-        <v>704254</v>
-      </c>
-      <c r="XK2">
-        <v>737251</v>
-      </c>
-      <c r="XL2">
-        <v>798662</v>
-      </c>
-      <c r="XM2">
-        <v>332579</v>
-      </c>
-      <c r="XN2">
-        <v>266513</v>
-      </c>
-      <c r="XO2">
-        <v>626043</v>
-      </c>
-      <c r="XP2">
-        <v>956291</v>
-      </c>
-      <c r="XQ2">
-        <v>866945</v>
-      </c>
-      <c r="XR2">
-        <v>186606</v>
-      </c>
-      <c r="XS2">
-        <v>505517</v>
-      </c>
-      <c r="XT2">
-        <v>1257581</v>
-      </c>
-      <c r="XU2">
-        <v>987398</v>
-      </c>
-      <c r="XV2">
-        <v>465879</v>
-      </c>
-      <c r="XW2">
-        <v>152017</v>
-      </c>
-      <c r="XX2">
-        <v>195160</v>
-      </c>
-      <c r="XY2">
-        <v>644552</v>
-      </c>
-      <c r="XZ2">
-        <v>43805</v>
-      </c>
-      <c r="YA2">
-        <v>1231988</v>
-      </c>
-      <c r="YB2">
-        <v>580925</v>
-      </c>
-      <c r="YC2">
-        <v>905630</v>
-      </c>
-      <c r="YD2">
-        <v>424474</v>
-      </c>
-      <c r="YE2">
-        <v>4536</v>
-      </c>
-      <c r="YF2">
-        <v>1006275</v>
-      </c>
-      <c r="YG2">
-        <v>231834</v>
-      </c>
-      <c r="YH2">
-        <v>193277</v>
-      </c>
-      <c r="YI2">
-        <v>96100</v>
-      </c>
-      <c r="YJ2">
-        <v>767455</v>
-      </c>
-      <c r="YK2">
-        <v>22902</v>
-      </c>
-      <c r="YL2">
-        <v>627652</v>
-      </c>
-      <c r="YM2">
-        <v>537325</v>
-      </c>
-      <c r="YN2">
-        <v>33939</v>
-      </c>
-      <c r="YO2">
-        <v>339821</v>
-      </c>
-      <c r="YP2">
-        <v>147420</v>
-      </c>
-      <c r="YQ2">
-        <v>59392</v>
-      </c>
-      <c r="YR2">
-        <v>677947</v>
-      </c>
-      <c r="YS2">
-        <v>545216</v>
-      </c>
-      <c r="YT2">
-        <v>936416</v>
-      </c>
-      <c r="YU2">
-        <v>664155</v>
-      </c>
-      <c r="YV2">
-        <v>812856</v>
-      </c>
-      <c r="YW2">
-        <v>596952</v>
-      </c>
-      <c r="YX2">
-        <v>434163</v>
-      </c>
-      <c r="YY2">
-        <v>780316</v>
-      </c>
-      <c r="YZ2">
-        <v>384249</v>
-      </c>
-      <c r="ZA2">
-        <v>1082579</v>
-      </c>
-      <c r="ZB2">
-        <v>940471</v>
-      </c>
-      <c r="ZC2">
-        <v>758648</v>
-      </c>
-      <c r="ZD2">
-        <v>299071</v>
-      </c>
-      <c r="ZE2">
-        <v>83155</v>
-      </c>
-      <c r="ZF2">
-        <v>736206</v>
-      </c>
-      <c r="ZG2">
-        <v>255081</v>
-      </c>
-      <c r="ZH2">
-        <v>1276756</v>
-      </c>
-      <c r="ZI2">
-        <v>30826</v>
-      </c>
-      <c r="ZJ2">
-        <v>485848</v>
-      </c>
-      <c r="ZK2">
-        <v>772135</v>
-      </c>
-      <c r="ZL2">
-        <v>582522</v>
-      </c>
-      <c r="ZM2">
-        <v>707292</v>
-      </c>
-      <c r="ZN2">
-        <v>610131</v>
-      </c>
-      <c r="ZO2">
-        <v>1090279</v>
-      </c>
-      <c r="ZP2">
-        <v>266395</v>
-      </c>
-      <c r="ZQ2">
-        <v>588678</v>
-      </c>
-      <c r="ZR2">
-        <v>206919</v>
-      </c>
-      <c r="ZS2">
-        <v>1266804</v>
-      </c>
-      <c r="ZT2">
-        <v>885035</v>
-      </c>
-      <c r="ZU2">
-        <v>448904</v>
-      </c>
-      <c r="ZV2">
-        <v>429181</v>
-      </c>
-      <c r="ZW2">
-        <v>313490</v>
-      </c>
-      <c r="ZX2">
-        <v>927928</v>
-      </c>
-      <c r="ZY2">
-        <v>1180957</v>
-      </c>
-      <c r="ZZ2">
-        <v>206027</v>
-      </c>
-      <c r="AAA2">
-        <v>556798</v>
-      </c>
-      <c r="AAB2">
-        <v>1043275</v>
-      </c>
-      <c r="AAC2">
-        <v>272877</v>
-      </c>
-      <c r="AAD2">
-        <v>106575</v>
-      </c>
-      <c r="AAE2">
-        <v>102412</v>
-      </c>
-      <c r="AAF2">
-        <v>1086418</v>
-      </c>
-      <c r="AAG2">
-        <v>236060</v>
-      </c>
-      <c r="AAH2">
-        <v>331281</v>
-      </c>
-      <c r="AAI2">
-        <v>1020773</v>
-      </c>
-      <c r="AAJ2">
-        <v>727425</v>
-      </c>
-      <c r="AAK2">
-        <v>1074142</v>
-      </c>
-      <c r="AAL2">
-        <v>1253229</v>
-      </c>
-      <c r="AAM2">
-        <v>121351</v>
-      </c>
-      <c r="AAN2">
-        <v>766927</v>
-      </c>
-      <c r="AAO2">
-        <v>183278</v>
-      </c>
-      <c r="AAP2">
-        <v>100105</v>
-      </c>
-      <c r="AAQ2">
-        <v>857367</v>
-      </c>
-      <c r="AAR2">
-        <v>288760</v>
-      </c>
-      <c r="AAS2">
-        <v>484903</v>
-      </c>
-      <c r="AAT2">
-        <v>224135</v>
-      </c>
-      <c r="AAU2">
-        <v>742550</v>
-      </c>
-      <c r="AAV2">
-        <v>127991</v>
-      </c>
-      <c r="AAW2">
-        <v>470350</v>
-      </c>
-      <c r="AAX2">
-        <v>460028</v>
-      </c>
-      <c r="AAY2">
-        <v>654928</v>
-      </c>
-      <c r="AAZ2">
-        <v>521710</v>
-      </c>
-      <c r="ABA2">
-        <v>35316</v>
-      </c>
-      <c r="ABB2">
-        <v>62158</v>
-      </c>
-      <c r="ABC2">
-        <v>454682</v>
-      </c>
-      <c r="ABD2">
-        <v>122286</v>
-      </c>
-      <c r="ABE2">
-        <v>718257</v>
-      </c>
-      <c r="ABF2">
-        <v>980681</v>
-      </c>
-      <c r="ABG2">
-        <v>405856</v>
-      </c>
-      <c r="ABH2">
-        <v>404420</v>
-      </c>
-      <c r="ABI2">
-        <v>28284</v>
-      </c>
-      <c r="ABJ2">
-        <v>12824</v>
-      </c>
-      <c r="ABK2">
-        <v>824162</v>
-      </c>
-      <c r="ABL2">
-        <v>909009</v>
-      </c>
-      <c r="ABM2">
-        <v>1154621</v>
-      </c>
-      <c r="ABN2">
-        <v>82350</v>
-      </c>
-      <c r="ABO2">
-        <v>65037</v>
-      </c>
-      <c r="ABP2">
-        <v>306624</v>
-      </c>
-      <c r="ABQ2">
-        <v>404932</v>
-      </c>
-      <c r="ABR2">
-        <v>1098961</v>
-      </c>
-      <c r="ABS2">
-        <v>566369</v>
-      </c>
-      <c r="ABT2">
-        <v>1213072</v>
-      </c>
-      <c r="ABU2">
-        <v>278646</v>
-      </c>
-      <c r="ABV2">
-        <v>231540</v>
-      </c>
-      <c r="ABW2">
-        <v>939842</v>
-      </c>
-      <c r="ABX2">
-        <v>64886</v>
-      </c>
-      <c r="ABY2">
-        <v>1160769</v>
-      </c>
-      <c r="ABZ2">
-        <v>425512</v>
-      </c>
-      <c r="ACA2">
-        <v>1263203</v>
-      </c>
-      <c r="ACB2">
-        <v>62354</v>
-      </c>
-      <c r="ACC2">
-        <v>1271419</v>
-      </c>
-      <c r="ACD2">
-        <v>836334</v>
-      </c>
-      <c r="ACE2">
-        <v>348827</v>
-      </c>
-      <c r="ACF2">
-        <v>1112181</v>
-      </c>
-      <c r="ACG2">
-        <v>377701</v>
-      </c>
-      <c r="ACH2">
-        <v>745841</v>
-      </c>
-      <c r="ACI2">
-        <v>513384</v>
-      </c>
-      <c r="ACJ2">
-        <v>1186947</v>
-      </c>
-      <c r="ACK2">
-        <v>845724</v>
-      </c>
-      <c r="ACL2">
-        <v>949302</v>
-      </c>
-      <c r="ACM2">
-        <v>527677</v>
-      </c>
-      <c r="ACN2">
-        <v>974281</v>
-      </c>
-      <c r="ACO2">
-        <v>661140</v>
-      </c>
-      <c r="ACP2">
-        <v>6502</v>
-      </c>
-      <c r="ACQ2">
-        <v>92403</v>
-      </c>
-      <c r="ACR2">
-        <v>53773</v>
-      </c>
-      <c r="ACS2">
-        <v>491662</v>
-      </c>
-      <c r="ACT2">
-        <v>864994</v>
-      </c>
-      <c r="ACU2">
-        <v>773938</v>
-      </c>
-      <c r="ACV2">
-        <v>1075051</v>
-      </c>
-      <c r="ACW2">
-        <v>337579</v>
-      </c>
-      <c r="ACX2">
-        <v>516080</v>
-      </c>
-      <c r="ACY2">
-        <v>634153</v>
-      </c>
-      <c r="ACZ2">
-        <v>1053126</v>
-      </c>
-      <c r="ADA2">
-        <v>346432</v>
-      </c>
-      <c r="ADB2">
-        <v>520716</v>
-      </c>
-      <c r="ADC2">
-        <v>176658</v>
-      </c>
-      <c r="ADD2">
-        <v>840738</v>
-      </c>
-      <c r="ADE2">
-        <v>215166</v>
-      </c>
-      <c r="ADF2">
-        <v>321548</v>
-      </c>
-      <c r="ADG2">
-        <v>278958</v>
-      </c>
-      <c r="ADH2">
-        <v>1221279</v>
-      </c>
-      <c r="ADI2">
-        <v>48650</v>
-      </c>
-      <c r="ADJ2">
-        <v>1122339</v>
-      </c>
-      <c r="ADK2">
-        <v>914834</v>
-      </c>
-      <c r="ADL2">
-        <v>428750</v>
-      </c>
-      <c r="ADM2">
-        <v>902110</v>
-      </c>
-      <c r="ADN2">
-        <v>574831</v>
-      </c>
-      <c r="ADO2">
-        <v>534135</v>
-      </c>
-      <c r="ADP2">
-        <v>1263193</v>
-      </c>
-      <c r="ADQ2">
-        <v>651473</v>
-      </c>
-      <c r="ADR2">
-        <v>461867</v>
-      </c>
-      <c r="ADS2">
-        <v>866142</v>
-      </c>
-      <c r="ADT2">
-        <v>994725</v>
-      </c>
-      <c r="ADU2">
-        <v>1216551</v>
-      </c>
-      <c r="ADV2">
-        <v>88119</v>
-      </c>
-      <c r="ADW2">
-        <v>1224519</v>
-      </c>
-      <c r="ADX2">
-        <v>881639</v>
-      </c>
-      <c r="ADY2">
-        <v>45292</v>
-      </c>
-      <c r="ADZ2">
-        <v>950685</v>
-      </c>
-      <c r="AEA2">
-        <v>584549</v>
-      </c>
-      <c r="AEB2">
-        <v>348817</v>
-      </c>
-      <c r="AEC2">
-        <v>475442</v>
-      </c>
-      <c r="AED2">
-        <v>659097</v>
-      </c>
-      <c r="AEE2">
-        <v>1238522</v>
-      </c>
-      <c r="AEF2">
-        <v>157000</v>
-      </c>
-      <c r="AEG2">
-        <v>1206424</v>
-      </c>
-      <c r="AEH2">
-        <v>89912</v>
-      </c>
-      <c r="AEI2">
-        <v>218594</v>
-      </c>
-      <c r="AEJ2">
-        <v>513421</v>
-      </c>
-      <c r="AEK2">
-        <v>439373</v>
-      </c>
-      <c r="AEL2">
-        <v>1125812</v>
-      </c>
-      <c r="AEM2">
-        <v>573696</v>
-      </c>
-      <c r="AEN2">
-        <v>671699</v>
-      </c>
-      <c r="AEO2">
-        <v>202106</v>
-      </c>
-      <c r="AEP2">
-        <v>1061323</v>
-      </c>
-      <c r="AEQ2">
-        <v>303395</v>
-      </c>
-      <c r="AER2">
-        <v>1164532</v>
-      </c>
-      <c r="AES2">
-        <v>283213</v>
-      </c>
-      <c r="AET2">
-        <v>310183</v>
-      </c>
-      <c r="AEU2">
-        <v>1118338</v>
-      </c>
-      <c r="AEV2">
-        <v>1180000</v>
-      </c>
-      <c r="AEW2">
-        <v>1286948</v>
-      </c>
-      <c r="AEX2">
-        <v>1161588</v>
-      </c>
-      <c r="AEY2">
-        <v>16868</v>
-      </c>
-      <c r="AEZ2">
-        <v>367930</v>
-      </c>
-      <c r="AFA2">
-        <v>182042</v>
-      </c>
-      <c r="AFB2">
-        <v>916924</v>
-      </c>
-      <c r="AFC2">
-        <v>1254644</v>
-      </c>
-      <c r="AFD2">
-        <v>108539</v>
-      </c>
-      <c r="AFE2">
-        <v>432561</v>
-      </c>
-      <c r="AFF2">
-        <v>716838</v>
-      </c>
-      <c r="AFG2">
-        <v>714393</v>
-      </c>
-      <c r="AFH2">
-        <v>704156</v>
-      </c>
-      <c r="AFI2">
-        <v>447541</v>
-      </c>
-      <c r="AFJ2">
-        <v>1273960</v>
-      </c>
-      <c r="AFK2">
-        <v>161576</v>
-      </c>
-      <c r="AFL2">
-        <v>511369</v>
-      </c>
-      <c r="AFM2">
-        <v>811690</v>
-      </c>
-      <c r="AFN2">
-        <v>665925</v>
-      </c>
-      <c r="AFO2">
-        <v>632458</v>
-      </c>
-      <c r="AFP2">
-        <v>559352</v>
-      </c>
-      <c r="AFQ2">
-        <v>29965</v>
-      </c>
-      <c r="AFR2">
-        <v>1021906</v>
-      </c>
-      <c r="AFS2">
-        <v>531602</v>
-      </c>
-      <c r="AFT2">
-        <v>570258</v>
-      </c>
-      <c r="AFU2">
-        <v>108543</v>
-      </c>
-      <c r="AFV2">
-        <v>362703</v>
-      </c>
-      <c r="AFW2">
-        <v>775783</v>
-      </c>
-      <c r="AFX2">
-        <v>1202765</v>
-      </c>
-      <c r="AFY2">
-        <v>495298</v>
-      </c>
-      <c r="AFZ2">
-        <v>1026948</v>
-      </c>
-      <c r="AGA2">
-        <v>548631</v>
-      </c>
-      <c r="AGB2">
-        <v>1035021</v>
-      </c>
-      <c r="AGC2">
-        <v>270210</v>
-      </c>
-      <c r="AGD2">
-        <v>229004</v>
-      </c>
-      <c r="AGE2">
-        <v>154520</v>
-      </c>
-      <c r="AGF2">
-        <v>523202</v>
-      </c>
-      <c r="AGG2">
-        <v>760549</v>
-      </c>
-      <c r="AGH2">
-        <v>483247</v>
-      </c>
-      <c r="AGI2">
-        <v>75029</v>
-      </c>
-      <c r="AGJ2">
-        <v>983797</v>
-      </c>
-      <c r="AGK2">
-        <v>80062</v>
-      </c>
-      <c r="AGL2">
-        <v>387775</v>
-      </c>
-      <c r="AGM2">
-        <v>1000430</v>
-      </c>
-      <c r="AGN2">
-        <v>789496</v>
-      </c>
-      <c r="AGO2">
-        <v>401796</v>
-      </c>
-      <c r="AGP2">
-        <v>140489</v>
-      </c>
-      <c r="AGQ2">
-        <v>105259</v>
-      </c>
-      <c r="AGR2">
-        <v>1191999</v>
-      </c>
-      <c r="AGS2">
-        <v>157928</v>
-      </c>
-      <c r="AGT2">
-        <v>591599</v>
-      </c>
-      <c r="AGU2">
-        <v>120822</v>
-      </c>
-      <c r="AGV2">
-        <v>335795</v>
-      </c>
-      <c r="AGW2">
-        <v>162440</v>
-      </c>
-      <c r="AGX2">
-        <v>227213</v>
-      </c>
-      <c r="AGY2">
-        <v>1228557</v>
-      </c>
-      <c r="AGZ2">
-        <v>130058</v>
-      </c>
-      <c r="AHA2">
-        <v>301031</v>
-      </c>
-      <c r="AHB2">
-        <v>5215</v>
-      </c>
-      <c r="AHC2">
-        <v>842217</v>
-      </c>
-      <c r="AHD2">
-        <v>378429</v>
-      </c>
-      <c r="AHE2">
-        <v>17393</v>
-      </c>
-      <c r="AHF2">
-        <v>888059</v>
-      </c>
-      <c r="AHG2">
-        <v>124885</v>
-      </c>
-      <c r="AHH2">
-        <v>690388</v>
-      </c>
-      <c r="AHI2">
-        <v>574009</v>
-      </c>
-      <c r="AHJ2">
-        <v>147924</v>
-      </c>
-      <c r="AHK2">
-        <v>552302</v>
-      </c>
-      <c r="AHL2">
-        <v>170738</v>
-      </c>
-      <c r="AHM2">
-        <v>316453</v>
-      </c>
-      <c r="AHN2">
-        <v>381298</v>
-      </c>
-      <c r="AHO2">
-        <v>644027</v>
-      </c>
-      <c r="AHP2">
-        <v>383147</v>
-      </c>
-      <c r="AHQ2">
-        <v>792471</v>
-      </c>
-      <c r="AHR2">
-        <v>975357</v>
-      </c>
-      <c r="AHS2">
-        <v>706840</v>
-      </c>
-      <c r="AHT2">
-        <v>251687</v>
-      </c>
-      <c r="AHU2">
-        <v>40730</v>
-      </c>
-      <c r="AHV2">
-        <v>40257</v>
-      </c>
-      <c r="AHW2">
-        <v>960528</v>
-      </c>
-      <c r="AHX2">
-        <v>20086</v>
-      </c>
-      <c r="AHY2">
-        <v>729840</v>
-      </c>
-      <c r="AHZ2">
-        <v>298838</v>
-      </c>
-      <c r="AIA2">
-        <v>399304</v>
-      </c>
-      <c r="AIB2">
-        <v>487856</v>
-      </c>
-      <c r="AIC2">
-        <v>554527</v>
-      </c>
-      <c r="AID2">
-        <v>618009</v>
-      </c>
-      <c r="AIE2">
-        <v>1086388</v>
-      </c>
-      <c r="AIF2">
-        <v>909360</v>
-      </c>
-      <c r="AIG2">
-        <v>486624</v>
-      </c>
-      <c r="AIH2">
-        <v>481196</v>
-      </c>
-      <c r="AII2">
-        <v>585906</v>
-      </c>
-      <c r="AIJ2">
-        <v>515801</v>
-      </c>
-      <c r="AIK2">
-        <v>957345</v>
-      </c>
-      <c r="AIL2">
-        <v>38669</v>
-      </c>
-      <c r="AIM2">
-        <v>719203</v>
-      </c>
-      <c r="AIN2">
-        <v>1132071</v>
-      </c>
-      <c r="AIO2">
-        <v>1248574</v>
-      </c>
-      <c r="AIP2">
-        <v>1261622</v>
-      </c>
-      <c r="AIQ2">
-        <v>587377</v>
-      </c>
-      <c r="AIR2">
-        <v>902569</v>
-      </c>
-      <c r="AIS2">
-        <v>819561</v>
-      </c>
-      <c r="AIT2">
-        <v>76513</v>
-      </c>
-      <c r="AIU2">
-        <v>1170423</v>
-      </c>
-      <c r="AIV2">
-        <v>673594</v>
-      </c>
-      <c r="AIW2">
-        <v>19465</v>
-      </c>
-      <c r="AIX2">
-        <v>295349</v>
-      </c>
-      <c r="AIY2">
-        <v>895090</v>
-      </c>
-      <c r="AIZ2">
-        <v>748251</v>
-      </c>
-      <c r="AJA2">
-        <v>135547</v>
-      </c>
-      <c r="AJB2">
-        <v>104739</v>
-      </c>
-      <c r="AJC2">
-        <v>992350</v>
-      </c>
-      <c r="AJD2">
-        <v>681644</v>
-      </c>
-      <c r="AJE2">
-        <v>508647</v>
-      </c>
-      <c r="AJF2">
-        <v>607721</v>
-      </c>
-      <c r="AJG2">
-        <v>1023209</v>
-      </c>
-      <c r="AJH2">
-        <v>1129379</v>
-      </c>
-      <c r="AJI2">
-        <v>424605</v>
-      </c>
-      <c r="AJJ2">
-        <v>375930</v>
-      </c>
-      <c r="AJK2">
-        <v>417371</v>
-      </c>
-      <c r="AJL2">
-        <v>16241</v>
-      </c>
-      <c r="AJM2">
-        <v>1045670</v>
-      </c>
-      <c r="AJN2">
-        <v>25318</v>
-      </c>
-      <c r="AJO2">
-        <v>187524</v>
-      </c>
-      <c r="AJP2">
-        <v>463150</v>
-      </c>
-      <c r="AJQ2">
-        <v>540247</v>
-      </c>
-      <c r="AJR2">
-        <v>69627</v>
-      </c>
-      <c r="AJS2">
-        <v>621200</v>
-      </c>
-      <c r="AJT2">
-        <v>205263</v>
-      </c>
-      <c r="AJU2">
-        <v>89546</v>
-      </c>
-      <c r="AJV2">
-        <v>747429</v>
-      </c>
-      <c r="AJW2">
-        <v>440835</v>
-      </c>
-      <c r="AJX2">
-        <v>830493</v>
-      </c>
-      <c r="AJY2">
-        <v>184664</v>
-      </c>
-      <c r="AJZ2">
-        <v>319547</v>
-      </c>
-      <c r="AKA2">
-        <v>207857</v>
-      </c>
-      <c r="AKB2">
-        <v>365236</v>
-      </c>
-      <c r="AKC2">
-        <v>820608</v>
-      </c>
-      <c r="AKD2">
-        <v>244016</v>
-      </c>
-      <c r="AKE2">
-        <v>756848</v>
-      </c>
-      <c r="AKF2">
-        <v>287661</v>
-      </c>
-      <c r="AKG2">
-        <v>151837</v>
-      </c>
-      <c r="AKH2">
-        <v>197737</v>
-      </c>
-      <c r="AKI2">
-        <v>823839</v>
-      </c>
-      <c r="AKJ2">
-        <v>478778</v>
-      </c>
-      <c r="AKK2">
-        <v>114589</v>
-      </c>
-      <c r="AKL2">
-        <v>967941</v>
-      </c>
-      <c r="AKM2">
-        <v>980500</v>
-      </c>
-      <c r="AKN2">
-        <v>1241237</v>
-      </c>
-      <c r="AKO2">
-        <v>1150643</v>
-      </c>
-      <c r="AKP2">
-        <v>201719</v>
-      </c>
-      <c r="AKQ2">
-        <v>771368</v>
-      </c>
-      <c r="AKR2">
-        <v>844326</v>
-      </c>
-      <c r="AKS2">
-        <v>173829</v>
-      </c>
-      <c r="AKT2">
-        <v>785515</v>
-      </c>
-      <c r="AKU2">
-        <v>4596</v>
-      </c>
-      <c r="AKV2">
-        <v>1148310</v>
-      </c>
-      <c r="AKW2">
-        <v>17970</v>
-      </c>
-      <c r="AKX2">
-        <v>281411</v>
-      </c>
-      <c r="AKY2">
-        <v>230439</v>
-      </c>
-      <c r="AKZ2">
-        <v>753186</v>
-      </c>
-      <c r="ALA2">
-        <v>244606</v>
-      </c>
-      <c r="ALB2">
-        <v>240709</v>
-      </c>
-      <c r="ALC2">
-        <v>1240936</v>
-      </c>
-      <c r="ALD2">
-        <v>582398</v>
-      </c>
-      <c r="ALE2">
-        <v>93897</v>
-      </c>
-      <c r="ALF2">
-        <v>249184</v>
-      </c>
-      <c r="ALG2">
-        <v>219566</v>
-      </c>
-      <c r="ALH2">
-        <v>631650</v>
-      </c>
-      <c r="ALI2">
-        <v>457304</v>
-      </c>
-      <c r="ALJ2">
-        <v>451876</v>
-      </c>
-      <c r="ALK2">
-        <v>605403</v>
-      </c>
-      <c r="ALL2">
-        <v>359947</v>
       </c>
     </row>
   </sheetData>

</xml_diff>